<commit_message>
planes y cuenta ajustes
</commit_message>
<xml_diff>
--- a/docs/cuentas/U-FT-12.010.069_Certificacion_determinacion_cedular_Rentas_de_Trabajo_V.6.1.1VF.xlsx
+++ b/docs/cuentas/U-FT-12.010.069_Certificacion_determinacion_cedular_Rentas_de_Trabajo_V.6.1.1VF.xlsx
@@ -2280,9 +2280,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>1428120</xdr:colOff>
+      <xdr:colOff>1427760</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>160920</xdr:rowOff>
+      <xdr:rowOff>160560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2296,7 +2296,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="11543760" y="133200"/>
-          <a:ext cx="2942640" cy="1542240"/>
+          <a:ext cx="2942280" cy="1541880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6487,7 +6487,7 @@
       </c>
       <c r="H17" s="76"/>
       <c r="I17" s="77" t="n">
-        <v>46078</v>
+        <v>46092</v>
       </c>
       <c r="J17" s="78"/>
       <c r="K17" s="2"/>
@@ -6952,7 +6952,7 @@
         <v>48</v>
       </c>
       <c r="C41" s="125" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="D41" s="126"/>
       <c r="E41" s="126"/>
@@ -6984,7 +6984,7 @@
         <v>50</v>
       </c>
       <c r="C42" s="125" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="D42" s="49"/>
       <c r="E42" s="49"/>

</xml_diff>

<commit_message>
chore: save remaining workspace changes
</commit_message>
<xml_diff>
--- a/docs/cuentas/U-FT-12.010.069_Certificacion_determinacion_cedular_Rentas_de_Trabajo_V.6.1.1VF.xlsx
+++ b/docs/cuentas/U-FT-12.010.069_Certificacion_determinacion_cedular_Rentas_de_Trabajo_V.6.1.1VF.xlsx
@@ -508,7 +508,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">3065-OSE-141-2025</t>
+    <t xml:space="preserve">3065-OSE-282-2025</t>
   </si>
   <si>
     <t xml:space="preserve">Aporte obligatorio a salud (12,5%)</t>
@@ -2280,9 +2280,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>1427040</xdr:colOff>
+      <xdr:colOff>1426680</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>159840</xdr:rowOff>
+      <xdr:rowOff>159480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2296,7 +2296,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="11543760" y="133200"/>
-          <a:ext cx="2941560" cy="1541160"/>
+          <a:ext cx="2941200" cy="1540800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6487,7 +6487,7 @@
       </c>
       <c r="H17" s="76"/>
       <c r="I17" s="77" t="n">
-        <v>46162</v>
+        <v>46224</v>
       </c>
       <c r="J17" s="78"/>
       <c r="K17" s="2"/>

</xml_diff>